<commit_message>
chore: cuentas.xlsx a plantilla vacia de 10 filas (modo registro)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cuentas.xlsx
+++ b/cuentas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,95 +447,645 @@
           <t>Puerto</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Modo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Cedula</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>PrimerNombre</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>PrimerApellido</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Telefono</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ExpedicionDD</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ExpedicionMM</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ExpedicionYYYY</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>NacimientoDD</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>NacimientoMM</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>NacimientoYYYY</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>LugarExpedicion</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>usuario_demo_01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>clave-ficticia-1</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nombre Demo 01</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>demo01@ejemplo.com</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>abcd efgh ijkl 0001</t>
-        </is>
-      </c>
+          <t>Cuenta 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>9222</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>usuario_demo_02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clave-ficticia-2</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Nombre Demo 02</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>demo02@ejemplo.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>abcd efgh ijkl 0002</t>
-        </is>
-      </c>
+          <t>Cuenta 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>9223</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>usuario_demo_03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>clave-ficticia-3</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nombre Demo 03</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>demo03@ejemplo.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>abcd efgh ijkl 0003</t>
-        </is>
-      </c>
+          <t>Cuenta 3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>9224</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cuenta 4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>9225</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cuenta 5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>9226</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Cuenta 6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>9227</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Cuenta 7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>9228</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Cuenta 8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>9229</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cuenta 9</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>9230</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cuenta 10</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>9231</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>registro</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>BOGOTA</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>